<commit_message>
Initial working NSE scraper
</commit_message>
<xml_diff>
--- a/exports/securities_below_20_2026-05-15.xlsx
+++ b/exports/securities_below_20_2026-05-15.xlsx
@@ -476,22 +476,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4.86</t>
+          <t>4.78</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>16.55</t>
+          <t>14.63</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>29,88,525</t>
+          <t>41,32,860</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>146.74</t>
+          <t>202.92</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -528,22 +528,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.90</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>12.66</t>
+          <t>13.92</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>7,66,819</t>
+          <t>11,72,275</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>6.67</t>
+          <t>10.32</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -580,22 +580,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>19.91</t>
+          <t>19.68</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>12.36</t>
+          <t>11.06</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>11,012</t>
+          <t>12,908</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2.17</t>
+          <t>2.54</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -607,567 +607,567 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FMNL</t>
+          <t>HYBRIDFIN</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.87</t>
+          <t>18.95</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>11.58</t>
+          <t>19.90</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10.62</t>
+          <t>17.42</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.53</t>
+          <t>18.19</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>11.50</t>
+          <t>19.90</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9.21</t>
+          <t>9.40</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1,07,546</t>
+          <t>10,985</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>11.92</t>
+          <t>2.09</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>22-Oct-2024</t>
+          <t>19-Jul-2024</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>EFCIL-RE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>15.20</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15.63</t>
+          <t>17.50</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>14.46</t>
+          <t>11.50</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14.39</t>
+          <t>15.06</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>15.35</t>
+          <t>16.11</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6.67</t>
+          <t>6.97</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1,77,156</t>
+          <t>2,81,875</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>26.96</t>
+          <t>38.48</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>18-Sep-2014</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TECILCHEM</t>
+          <t>JPPOWER</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>12.03</t>
+          <t>17.84</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>12.84</t>
+          <t>20.38</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>12.00</t>
+          <t>17.43</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>11.96</t>
+          <t>17.86</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>12.70</t>
+          <t>18.95</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6.19</t>
+          <t>6.10</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>5,332</t>
+          <t>73,80,85,898</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0.66</t>
+          <t>1,43,852.94</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>19-Sep-2024</t>
+          <t>26-Aug-2024</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CINEVISTA</t>
+          <t>CREATIVEYE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15.50</t>
+          <t>6.89</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16.50</t>
+          <t>7.10</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>15.02</t>
+          <t>6.62</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>15.43</t>
+          <t>6.69</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>16.38</t>
+          <t>7.08</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6.16</t>
+          <t>5.83</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>29,597</t>
+          <t>13,517</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.74</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>13-Sep-2024</t>
+          <t>23-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>RMDRIP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>12.45</t>
+          <t>18.50</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.13</t>
+          <t>19.33</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>12.04</t>
+          <t>18.15</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>12.21</t>
+          <t>18.41</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.85</t>
+          <t>19.33</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>5.00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>63,243</t>
+          <t>8,13,608</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>8.06</t>
+          <t>154.26</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>20-Sep-2024</t>
+          <t>10-Apr-2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RMDRIP</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.50</t>
+          <t>4.92</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>19.33</t>
+          <t>5.06</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>18.15</t>
+          <t>4.60</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.41</t>
+          <t>4.82</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>19.33</t>
+          <t>5.06</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5.00</t>
+          <t>4.98</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>7,81,826</t>
+          <t>34,746</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>148.08</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>10-Apr-2026</t>
+          <t>04-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t>13.68</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.59</t>
+          <t>14.16</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>13.49</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>13.49</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1.59</t>
+          <t>14.16</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4.61</t>
+          <t>4.97</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>29,606</t>
+          <t>14,664</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0.46</t>
+          <t>2.04</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>17-Sep-2024</t>
+          <t>25-Jun-2024</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>DRCSYSTEMS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>15.49</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>14.62</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>14.79</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>15.49</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4.52</t>
+          <t>4.73</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>18,548</t>
+          <t>73,097</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>0.29</t>
+          <t>11.04</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>17-Sep-2024</t>
+          <t>09-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ORTINGLOBE</t>
+          <t>SADBHIN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.57</t>
+          <t>2.73</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15.25</t>
+          <t>2.85</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>14.31</t>
+          <t>2.63</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14.60</t>
+          <t>2.73</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>15.25</t>
+          <t>2.85</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4.45</t>
+          <t>4.40</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>17,713</t>
+          <t>2,08,623</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>5.59</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>22-Sep-2023</t>
+          <t>23-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RRIL</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>19.40</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>19.90</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>18.66</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>19.02</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>19.85</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4.36</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>17,848</t>
+          <t>2,93,89,462</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>3.52</t>
+          <t>70.53</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>4.95</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>4.76</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>4.95</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4.17</t>
+          <t>3.99</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1,60,71,787</t>
+          <t>1,31,883</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>38.57</t>
+          <t>6.44</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1179,208 +1179,208 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AIRAN</t>
+          <t>BANK10ADD</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>16.40</t>
+          <t>16.04</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17.50</t>
+          <t>16.65</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>16.25</t>
+          <t>16.02</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>16.43</t>
+          <t>16.04</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>17.10</t>
+          <t>16.65</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4.08</t>
+          <t>3.80</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>64,361</t>
+          <t>63,30,090</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>11.08</t>
+          <t>1,024.84</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>14-Aug-2019</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KHANDSE</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>17.45</t>
+          <t>7.07</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17.45</t>
+          <t>7.25</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>16.35</t>
+          <t>6.90</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>16.32</t>
+          <t>6.99</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>16.98</t>
+          <t>7.25</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>3.72</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1,353</t>
+          <t>46,227</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>3.24</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>19-Sep-2024</t>
+          <t>23-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>ASHIMASYN</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0.53</t>
+          <t>17.00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>17.90</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>16.36</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>17.00</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>17.60</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>3.85</t>
+          <t>3.53</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>5,81,421</t>
+          <t>2,80,492</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>3.08</t>
+          <t>48.69</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>28-Apr-2025</t>
+          <t>11-Aug-2022</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>URJA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>10.60</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>11.25</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.53</t>
+          <t>10.50</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0.53</t>
+          <t>10.67</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>10.98</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>3.77</t>
+          <t>2.91</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>4,41,145</t>
+          <t>20,59,718</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.43</t>
+          <t>222.66</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>17-Sep-2024</t>
+          <t>21-Aug-2024</t>
         </is>
       </c>
     </row>
@@ -1412,22 +1412,22 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>6.79</t>
+          <t>6.74</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>3.66</t>
+          <t>2.90</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>33,504</t>
+          <t>39,527</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>2.67</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1439,99 +1439,99 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PAVNAIND</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>18.96</t>
+          <t>1.53</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>19.89</t>
+          <t>1.59</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>18.91</t>
+          <t>1.50</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>18.98</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>19.64</t>
+          <t>1.56</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>2.63</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>46,476</t>
+          <t>33,613</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>9.16</t>
+          <t>0.52</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>01-Sep-2025</t>
+          <t>17-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EFCIL-RE</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>15.00</t>
+          <t>8.28</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>15.00</t>
+          <t>8.28</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>12.50</t>
+          <t>7.75</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>15.06</t>
+          <t>8.59</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>13.00</t>
+          <t>7.80</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.68</t>
+          <t>-9.20</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1,66,273</t>
+          <t>7,58,488</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>22.70</t>
+          <t>59.84</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1543,988 +1543,988 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>ABINFRA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>8.28</t>
+          <t>14.05</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>8.28</t>
+          <t>14.05</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>7.78</t>
+          <t>13.01</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>8.59</t>
+          <t>13.90</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>7.88</t>
+          <t>13.11</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>-8.27</t>
+          <t>-5.68</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>3,72,173</t>
+          <t>3,87,017</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>29.66</t>
+          <t>51.82</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17-Oct-2025</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AONESILVER</t>
+          <t>KRIDHANINF</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10.45</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>10.45</t>
+          <t>3.12</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10.04</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>10.76</t>
+          <t>3.02</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>10.14</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>-5.76</t>
+          <t>-4.97</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>10,49,514</t>
+          <t>78,935</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>107.37</t>
+          <t>2.28</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23-Sep-2022</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GRADIENTE</t>
+          <t>KESORAMIND</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>6.93</t>
+          <t>13.07</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>6.93</t>
+          <t>13.24</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>6.93</t>
+          <t>12.30</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>7.29</t>
+          <t>12.94</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>6.93</t>
+          <t>12.30</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>-4.94</t>
+          <t>-4.95</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>17,693</t>
+          <t>74,77,517</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>927.21</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10-Mar-2025</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PARSVNATH</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>6.93</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>6.93</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>6.93</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>5.68</t>
+          <t>7.29</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>6.93</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>-4.93</t>
+          <t>-4.94</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1,55,304</t>
+          <t>18,715</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>8.39</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>20-Sep-2024</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>PARSVNATH</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>5.40</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>5.40</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3.93</t>
+          <t>5.40</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>5.68</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>3.93</t>
+          <t>5.40</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>-4.84</t>
+          <t>-4.93</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>10,45,198</t>
+          <t>2,42,045</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>43.06</t>
+          <t>13.07</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>18-Jun-2024</t>
+          <t>20-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>4.73</t>
+          <t>7.71</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>4.98</t>
+          <t>7.93</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>4.73</t>
+          <t>7.55</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>4.97</t>
+          <t>7.94</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>4.73</t>
+          <t>7.55</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>-4.83</t>
+          <t>-4.91</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>3,339</t>
+          <t>39,917</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>3.04</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>17-Sep-2024</t>
+          <t>05-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>4.96</t>
+          <t>11.51</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>4.96</t>
+          <t>11.54</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4.74</t>
+          <t>10.96</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>4.98</t>
+          <t>11.63</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>4.74</t>
+          <t>11.06</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>-4.82</t>
+          <t>-4.90</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>4,23,508</t>
+          <t>2,91,223</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>20.20</t>
+          <t>32.33</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>12-Sep-2024</t>
+          <t>12-Dec-2024</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2.29</t>
+          <t>4.15</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2.29</t>
+          <t>4.15</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2.18</t>
+          <t>3.93</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2.29</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2.18</t>
+          <t>3.93</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>-4.80</t>
+          <t>-4.84</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>3,65,872</t>
+          <t>10,93,390</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>8.12</t>
+          <t>45.05</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>20-Sep-2024</t>
+          <t>18-Jun-2024</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>KESORAMIND</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>13.07</t>
+          <t>4.73</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>13.24</t>
+          <t>4.98</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>12.30</t>
+          <t>4.73</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>12.94</t>
+          <t>4.97</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>12.35</t>
+          <t>4.73</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>-4.56</t>
+          <t>-4.83</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>64,33,240</t>
+          <t>5,453</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>798.37</t>
+          <t>0.26</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>10-Mar-2025</t>
+          <t>17-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>11.51</t>
+          <t>4.96</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11.54</t>
+          <t>4.96</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10.96</t>
+          <t>4.74</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>11.63</t>
+          <t>4.98</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>11.13</t>
+          <t>4.74</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>-4.30</t>
+          <t>-4.82</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2,19,669</t>
+          <t>5,80,292</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>24.41</t>
+          <t>27.62</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>12-Dec-2024</t>
+          <t>12-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BAIDFIN</t>
+          <t>MADHUCON</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>11.91</t>
+          <t>5.61</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11.98</t>
+          <t>5.89</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>11.46</t>
+          <t>5.33</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>11.91</t>
+          <t>5.61</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>11.46</t>
+          <t>5.34</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>-3.78</t>
+          <t>-4.81</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>31,674</t>
+          <t>47,397</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>3.70</t>
+          <t>2.68</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>17-Nov-2025</t>
+          <t>20-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>KRIDHANINF</t>
+          <t>SIL</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>16.25</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>3.12</t>
+          <t>16.38</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2.87</t>
+          <t>15.31</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>3.02</t>
+          <t>16.13</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2.91</t>
+          <t>15.36</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>-3.64</t>
+          <t>-4.77</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>59,090</t>
+          <t>32,107</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>1.71</t>
+          <t>5.07</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>23-Sep-2022</t>
+          <t>20-Feb-2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ACCURACY</t>
+          <t>GAYAPROJ</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>5.90</t>
+          <t>18.80</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>5.99</t>
+          <t>18.80</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5.70</t>
+          <t>18.02</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>5.99</t>
+          <t>18.96</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>5.78</t>
+          <t>18.09</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>-3.51</t>
+          <t>-4.59</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1,68,255</t>
+          <t>2,96,585</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>9.69</t>
+          <t>53.83</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>15-Feb-2023</t>
+          <t>15-Sep-2021</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>EASEMYTRIP</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>18.80</t>
+          <t>8.24</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>18.80</t>
+          <t>8.24</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>18.05</t>
+          <t>7.80</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>18.96</t>
+          <t>8.27</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>18.40</t>
+          <t>7.90</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>-2.95</t>
+          <t>-4.47</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1,25,609</t>
+          <t>1,11,65,755</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>22.97</t>
+          <t>897.73</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>15-Sep-2021</t>
+          <t>29-Nov-2024</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GVPTECH</t>
+          <t>GANGAFORGE</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>6.71</t>
+          <t>2.55</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>6.92</t>
+          <t>2.60</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>6.60</t>
+          <t>2.30</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>6.86</t>
+          <t>2.46</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>6.66</t>
+          <t>2.35</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>-2.92</t>
+          <t>-4.47</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>46,630</t>
+          <t>13,63,418</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>32.86</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>11-Jul-2025</t>
+          <t>20-Sep-2021</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABINFRA</t>
+          <t>ACCURACY</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>14.05</t>
+          <t>5.90</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14.05</t>
+          <t>5.99</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>13.52</t>
+          <t>5.70</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>13.90</t>
+          <t>5.99</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>13.52</t>
+          <t>5.73</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>-2.73</t>
+          <t>-4.34</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1,23,795</t>
+          <t>2,20,632</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>16.95</t>
+          <t>12.71</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>17-Oct-2025</t>
+          <t>15-Feb-2023</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MKPL</t>
+          <t>SUBEXLTD</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>5.29</t>
+          <t>10.98</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>5.29</t>
+          <t>10.98</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>5.10</t>
+          <t>10.40</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>10.91</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>5.10</t>
+          <t>10.45</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>-2.67</t>
+          <t>-4.22</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1,13,023</t>
+          <t>9,04,598</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>5.82</t>
+          <t>95.53</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>23-Sep-2024</t>
+          <t>29-Jul-2024</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ARCHIES</t>
+          <t>IBULLSLTD</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>14.50</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>15.70</t>
+          <t>20.16</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>14.28</t>
+          <t>19.02</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>14.70</t>
+          <t>19.98</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>14.32</t>
+          <t>19.20</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>-2.59</t>
+          <t>-3.90</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>22,021</t>
+          <t>57,30,626</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>1,106.58</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>17-Sep-2024</t>
+          <t>19-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GLOBALE</t>
+          <t>AONESILVER</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>13.40</t>
+          <t>10.45</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>13.42</t>
+          <t>10.45</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>13.14</t>
+          <t>10.04</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>13.50</t>
+          <t>10.76</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>13.16</t>
+          <t>10.35</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>-2.52</t>
+          <t>-3.81</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>3,293</t>
+          <t>16,29,685</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>0.44</t>
+          <t>166.06</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>23-Sep-2024</t>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>